<commit_message>
WIP: save changes before rebase
</commit_message>
<xml_diff>
--- a/withoutOutofDomain_samePrompt_25_6/test_case/output_11_6/category_classi_result.xlsx
+++ b/withoutOutofDomain_samePrompt_25_6/test_case/output_11_6/category_classi_result.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\seniorProject\term2\output_11_6\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\update_project\withoutOutofDomain_samePrompt_25_6\test_case\output_11_6\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0993BA8-C66D-4CB3-80D4-2268F4C91EC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF8CA0FA-53FC-4295-88C3-3DD532289564}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="43080" yWindow="4605" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>